<commit_message>
Sincronizacion 2026-09-25: laminas nacionales, dimensiones, educacion y sexo-edad (FONASA/ISAPRE por sexo como tasas) y payloads
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_d_dep_a_2018_coquimbo.xlsx
+++ b/output/graficos_dimensiones/comunal_d_dep_a_2018_coquimbo.xlsx
@@ -57,6 +57,9 @@
     <t xml:space="preserve">Illapel</t>
   </si>
   <si>
+    <t xml:space="preserve">Paihuano</t>
+  </si>
+  <si>
     <t xml:space="preserve">Los Vilos</t>
   </si>
   <si>
@@ -75,9 +78,6 @@
     <t xml:space="preserve">Vicuña</t>
   </si>
   <si>
-    <t xml:space="preserve">Paihuano</t>
-  </si>
-  <si>
     <t xml:space="preserve">Campo</t>
   </si>
   <si>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-12 22:19</t>
+    <t xml:space="preserve">2026-09-23 23:48</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -636,7 +636,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>4203</v>
+        <v>4105</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>2018</v>
@@ -653,13 +653,13 @@
         <v>14</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>4204</v>
+        <v>4203</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>2018</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>59.7</v>
+        <v>59.82</v>
       </c>
     </row>
     <row r="11">
@@ -670,13 +670,13 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>4303</v>
+        <v>4204</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>2018</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>59.49</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="12">
@@ -687,13 +687,13 @@
         <v>16</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>4301</v>
+        <v>4303</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>2018</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>57.99</v>
+        <v>59.49</v>
       </c>
     </row>
     <row r="13">
@@ -704,13 +704,13 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>4101</v>
+        <v>4301</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>2018</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>56.55</v>
+        <v>57.99</v>
       </c>
     </row>
     <row r="14">
@@ -721,13 +721,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>4106</v>
+        <v>4101</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>2018</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>55.47</v>
+        <v>56.55</v>
       </c>
     </row>
     <row r="15">
@@ -735,16 +735,16 @@
         <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>4102</v>
+        <v>4106</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>2018</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>55.32</v>
+        <v>55.47</v>
       </c>
     </row>
     <row r="16">
@@ -752,13 +752,17 @@
         <v>5</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>4105</v>
-      </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+        <v>4102</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>55.32</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E16"/>

</xml_diff>